<commit_message>
cds hooks requirement mapping for client v 2.2.1
</commit_message>
<xml_diff>
--- a/lib/davinci_crd_test_kit/requirements/cds-hooks_3.0.0-ballot_requirements.xlsx
+++ b/lib/davinci_crd_test_kit/requirements/cds-hooks_3.0.0-ballot_requirements.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karlnaden/GlenViewAssociates/Inferno/hti-4/CRD 2.2.1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karlnaden/GlenViewAssociates/Inferno/source/davinci-crd-test-kit/lib/davinci_crd_test_kit/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47843495-5FAB-1B4F-9BC3-FEDD9C0192EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2569BB1-4C6D-1743-87B5-05DEC082AFC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="1320" windowWidth="33780" windowHeight="18000" activeTab="2" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
+    <workbookView xWindow="780" yWindow="1320" windowWidth="33780" windowHeight="18000" activeTab="1" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="9" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1476" uniqueCount="486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1476" uniqueCount="482">
   <si>
     <r>
       <rPr>
@@ -2899,25 +2899,13 @@
     <t>Test Implementation Ticket</t>
   </si>
   <si>
-    <t>ID-110</t>
-  </si>
-  <si>
     <t>ID-115</t>
   </si>
   <si>
-    <t>ID-112</t>
-  </si>
-  <si>
     <t>ID-114</t>
   </si>
   <si>
     <t>ID-116</t>
-  </si>
-  <si>
-    <t>ID-111</t>
-  </si>
-  <si>
-    <t>ID-113</t>
   </si>
 </sst>
 </file>
@@ -3412,6 +3400,9 @@
     <xf numFmtId="0" fontId="20" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -3426,9 +3417,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3795,14 +3783,14 @@
       <c r="C3" s="30"/>
     </row>
     <row r="4" spans="1:3" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="43" t="s">
         <v>291</v>
       </c>
       <c r="B4" s="31"/>
       <c r="C4" s="32"/>
     </row>
     <row r="5" spans="1:3" ht="258" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="43"/>
+      <c r="A5" s="44"/>
       <c r="B5" s="35"/>
       <c r="C5" s="30"/>
     </row>
@@ -3814,17 +3802,17 @@
       <c r="C6" s="24"/>
     </row>
     <row r="7" spans="1:3" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="44" t="s">
+      <c r="A7" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="45"/>
+      <c r="B7" s="46"/>
     </row>
     <row r="8" spans="1:3" ht="126" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="44"/>
-      <c r="B8" s="46"/>
+      <c r="A8" s="45"/>
+      <c r="B8" s="47"/>
     </row>
     <row r="9" spans="1:3" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="42"/>
+      <c r="A9" s="43"/>
       <c r="B9" s="34"/>
     </row>
     <row r="10" spans="1:3" ht="292" x14ac:dyDescent="0.2">
@@ -3973,7 +3961,7 @@
       <c r="X2" s="10"/>
       <c r="AB2" s="10"/>
     </row>
-    <row r="3" spans="1:34" ht="68" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:34" ht="51" x14ac:dyDescent="0.2">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -3996,7 +3984,7 @@
         <v>453</v>
       </c>
       <c r="P3" s="13" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="R3" s="13" t="s">
         <v>90</v>
@@ -4185,7 +4173,7 @@
         <v>455</v>
       </c>
       <c r="P9" s="13" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="X9" s="10"/>
       <c r="Y9" s="4"/>
@@ -4746,7 +4734,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="35" spans="1:18" ht="68" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:18" ht="34" x14ac:dyDescent="0.2">
       <c r="A35" s="6">
         <v>25</v>
       </c>
@@ -4769,7 +4757,7 @@
         <v>461</v>
       </c>
       <c r="P35" s="13" t="s">
-        <v>481</v>
+        <v>457</v>
       </c>
     </row>
     <row r="36" spans="1:18" ht="34" x14ac:dyDescent="0.2">
@@ -5180,7 +5168,7 @@
         <v>463</v>
       </c>
       <c r="P53" s="13" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="54" spans="1:18" ht="85" x14ac:dyDescent="0.2">
@@ -5438,7 +5426,7 @@
       </c>
       <c r="N63" s="8"/>
     </row>
-    <row r="64" spans="1:18" ht="68" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:18" ht="51" x14ac:dyDescent="0.2">
       <c r="A64" s="6">
         <v>51</v>
       </c>
@@ -5464,7 +5452,7 @@
         <v>466</v>
       </c>
       <c r="P64" s="13" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
     </row>
     <row r="65" spans="1:16" ht="34" x14ac:dyDescent="0.2">
@@ -5518,7 +5506,7 @@
         <v>467</v>
       </c>
       <c r="P66" s="13" t="s">
-        <v>484</v>
+        <v>457</v>
       </c>
     </row>
     <row r="67" spans="1:16" ht="85" x14ac:dyDescent="0.2">
@@ -5732,7 +5720,7 @@
       <c r="N76" s="8"/>
       <c r="O76" s="8"/>
     </row>
-    <row r="77" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:16" ht="51" x14ac:dyDescent="0.2">
       <c r="A77" s="6">
         <v>239</v>
       </c>
@@ -5758,7 +5746,7 @@
         <v>477</v>
       </c>
       <c r="P77" s="13" t="s">
-        <v>485</v>
+        <v>457</v>
       </c>
     </row>
     <row r="78" spans="1:16" ht="68" x14ac:dyDescent="0.2">
@@ -5984,7 +5972,7 @@
         <v>463</v>
       </c>
       <c r="P86" s="13" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="87" spans="1:18" ht="85" x14ac:dyDescent="0.2">
@@ -6016,7 +6004,7 @@
         <v>463</v>
       </c>
       <c r="P87" s="13" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="88" spans="1:18" ht="51" x14ac:dyDescent="0.2">
@@ -9044,7 +9032,7 @@
         <v>471</v>
       </c>
       <c r="P206" s="13" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
     </row>
     <row r="207" spans="1:18" ht="51" x14ac:dyDescent="0.2">
@@ -9136,7 +9124,7 @@
         <v>472</v>
       </c>
       <c r="P210" s="13" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
     </row>
     <row r="211" spans="1:16" ht="85" x14ac:dyDescent="0.2">
@@ -9165,7 +9153,7 @@
         <v>463</v>
       </c>
       <c r="P211" s="13" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="212" spans="1:16" ht="102" x14ac:dyDescent="0.2">
@@ -10974,14 +10962,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="42" t="s">
         <v>290</v>
       </c>
-      <c r="B1" s="47"/>
+      <c r="B1" s="42"/>
     </row>
     <row r="2" spans="1:2" ht="82" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="47"/>
-      <c r="B2" s="47"/>
+      <c r="A2" s="42"/>
+      <c r="B2" s="42"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="15" t="s">
@@ -11208,6 +11196,19 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="b5a44311-ed64-4a72-909f-c9dc6973bde2" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Description xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
+    <SortOrder xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC335ED7BB179244BF94A0DFE64544DC" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d3a0f66abe5d2a0564332877ab55d3f7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="eebd8b74-b9de-41b2-9247-c010c4973c2b" xmlns:ns3="b7009bbd-f938-489b-a530-f05273710fff" xmlns:ns4="b5a44311-ed64-4a72-909f-c9dc6973bde2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ec7ca2ee893ff8a0f61d4046c6461645" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="eebd8b74-b9de-41b2-9247-c010c4973c2b"/>
@@ -11461,19 +11462,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="b5a44311-ed64-4a72-909f-c9dc6973bde2" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Description xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
-    <SortOrder xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA84097F-5807-4DCF-92C6-48C9EE26CFB8}">
   <ds:schemaRefs>
@@ -11483,6 +11471,24 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19B0E317-5E0E-4728-AB3F-40F2C2B957FB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="b5a44311-ed64-4a72-909f-c9dc6973bde2"/>
+    <ds:schemaRef ds:uri="b7009bbd-f938-489b-a530-f05273710fff"/>
+    <ds:schemaRef ds:uri="eebd8b74-b9de-41b2-9247-c010c4973c2b"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BFE547E3-BD0E-4C13-B5EC-CA56CC895052}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11500,22 +11506,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19B0E317-5E0E-4728-AB3F-40F2C2B957FB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="b5a44311-ed64-4a72-909f-c9dc6973bde2"/>
-    <ds:schemaRef ds:uri="b7009bbd-f938-489b-a530-f05273710fff"/>
-    <ds:schemaRef ds:uri="eebd8b74-b9de-41b2-9247-c010c4973c2b"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
ID-82: CRD Client Suite v221 requirements mapping (#78)
* cds hooks requirement mapping for client v 2.2.1

* crd client v221 requirements mapping

* add us core sets, generate coverage

* fix added requirements
</commit_message>
<xml_diff>
--- a/lib/davinci_crd_test_kit/requirements/cds-hooks_3.0.0-ballot_requirements.xlsx
+++ b/lib/davinci_crd_test_kit/requirements/cds-hooks_3.0.0-ballot_requirements.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karlnaden/GlenViewAssociates/Inferno/hti-4/CRD 2.2.1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karlnaden/GlenViewAssociates/Inferno/source/davinci-crd-test-kit/lib/davinci_crd_test_kit/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47843495-5FAB-1B4F-9BC3-FEDD9C0192EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2569BB1-4C6D-1743-87B5-05DEC082AFC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="1320" windowWidth="33780" windowHeight="18000" activeTab="2" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
+    <workbookView xWindow="780" yWindow="1320" windowWidth="33780" windowHeight="18000" activeTab="1" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="9" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1476" uniqueCount="486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1476" uniqueCount="482">
   <si>
     <r>
       <rPr>
@@ -2899,25 +2899,13 @@
     <t>Test Implementation Ticket</t>
   </si>
   <si>
-    <t>ID-110</t>
-  </si>
-  <si>
     <t>ID-115</t>
   </si>
   <si>
-    <t>ID-112</t>
-  </si>
-  <si>
     <t>ID-114</t>
   </si>
   <si>
     <t>ID-116</t>
-  </si>
-  <si>
-    <t>ID-111</t>
-  </si>
-  <si>
-    <t>ID-113</t>
   </si>
 </sst>
 </file>
@@ -3412,6 +3400,9 @@
     <xf numFmtId="0" fontId="20" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -3426,9 +3417,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3795,14 +3783,14 @@
       <c r="C3" s="30"/>
     </row>
     <row r="4" spans="1:3" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="43" t="s">
         <v>291</v>
       </c>
       <c r="B4" s="31"/>
       <c r="C4" s="32"/>
     </row>
     <row r="5" spans="1:3" ht="258" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="43"/>
+      <c r="A5" s="44"/>
       <c r="B5" s="35"/>
       <c r="C5" s="30"/>
     </row>
@@ -3814,17 +3802,17 @@
       <c r="C6" s="24"/>
     </row>
     <row r="7" spans="1:3" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="44" t="s">
+      <c r="A7" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="45"/>
+      <c r="B7" s="46"/>
     </row>
     <row r="8" spans="1:3" ht="126" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="44"/>
-      <c r="B8" s="46"/>
+      <c r="A8" s="45"/>
+      <c r="B8" s="47"/>
     </row>
     <row r="9" spans="1:3" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="42"/>
+      <c r="A9" s="43"/>
       <c r="B9" s="34"/>
     </row>
     <row r="10" spans="1:3" ht="292" x14ac:dyDescent="0.2">
@@ -3973,7 +3961,7 @@
       <c r="X2" s="10"/>
       <c r="AB2" s="10"/>
     </row>
-    <row r="3" spans="1:34" ht="68" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:34" ht="51" x14ac:dyDescent="0.2">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -3996,7 +3984,7 @@
         <v>453</v>
       </c>
       <c r="P3" s="13" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
       <c r="R3" s="13" t="s">
         <v>90</v>
@@ -4185,7 +4173,7 @@
         <v>455</v>
       </c>
       <c r="P9" s="13" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="X9" s="10"/>
       <c r="Y9" s="4"/>
@@ -4746,7 +4734,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="35" spans="1:18" ht="68" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:18" ht="34" x14ac:dyDescent="0.2">
       <c r="A35" s="6">
         <v>25</v>
       </c>
@@ -4769,7 +4757,7 @@
         <v>461</v>
       </c>
       <c r="P35" s="13" t="s">
-        <v>481</v>
+        <v>457</v>
       </c>
     </row>
     <row r="36" spans="1:18" ht="34" x14ac:dyDescent="0.2">
@@ -5180,7 +5168,7 @@
         <v>463</v>
       </c>
       <c r="P53" s="13" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="54" spans="1:18" ht="85" x14ac:dyDescent="0.2">
@@ -5438,7 +5426,7 @@
       </c>
       <c r="N63" s="8"/>
     </row>
-    <row r="64" spans="1:18" ht="68" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:18" ht="51" x14ac:dyDescent="0.2">
       <c r="A64" s="6">
         <v>51</v>
       </c>
@@ -5464,7 +5452,7 @@
         <v>466</v>
       </c>
       <c r="P64" s="13" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
     </row>
     <row r="65" spans="1:16" ht="34" x14ac:dyDescent="0.2">
@@ -5518,7 +5506,7 @@
         <v>467</v>
       </c>
       <c r="P66" s="13" t="s">
-        <v>484</v>
+        <v>457</v>
       </c>
     </row>
     <row r="67" spans="1:16" ht="85" x14ac:dyDescent="0.2">
@@ -5732,7 +5720,7 @@
       <c r="N76" s="8"/>
       <c r="O76" s="8"/>
     </row>
-    <row r="77" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:16" ht="51" x14ac:dyDescent="0.2">
       <c r="A77" s="6">
         <v>239</v>
       </c>
@@ -5758,7 +5746,7 @@
         <v>477</v>
       </c>
       <c r="P77" s="13" t="s">
-        <v>485</v>
+        <v>457</v>
       </c>
     </row>
     <row r="78" spans="1:16" ht="68" x14ac:dyDescent="0.2">
@@ -5984,7 +5972,7 @@
         <v>463</v>
       </c>
       <c r="P86" s="13" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="87" spans="1:18" ht="85" x14ac:dyDescent="0.2">
@@ -6016,7 +6004,7 @@
         <v>463</v>
       </c>
       <c r="P87" s="13" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="88" spans="1:18" ht="51" x14ac:dyDescent="0.2">
@@ -9044,7 +9032,7 @@
         <v>471</v>
       </c>
       <c r="P206" s="13" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
     </row>
     <row r="207" spans="1:18" ht="51" x14ac:dyDescent="0.2">
@@ -9136,7 +9124,7 @@
         <v>472</v>
       </c>
       <c r="P210" s="13" t="s">
-        <v>479</v>
+        <v>457</v>
       </c>
     </row>
     <row r="211" spans="1:16" ht="85" x14ac:dyDescent="0.2">
@@ -9165,7 +9153,7 @@
         <v>463</v>
       </c>
       <c r="P211" s="13" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="212" spans="1:16" ht="102" x14ac:dyDescent="0.2">
@@ -10974,14 +10962,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="42" t="s">
         <v>290</v>
       </c>
-      <c r="B1" s="47"/>
+      <c r="B1" s="42"/>
     </row>
     <row r="2" spans="1:2" ht="82" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="47"/>
-      <c r="B2" s="47"/>
+      <c r="A2" s="42"/>
+      <c r="B2" s="42"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="15" t="s">
@@ -11208,6 +11196,19 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="b5a44311-ed64-4a72-909f-c9dc6973bde2" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Description xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
+    <SortOrder xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC335ED7BB179244BF94A0DFE64544DC" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d3a0f66abe5d2a0564332877ab55d3f7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="eebd8b74-b9de-41b2-9247-c010c4973c2b" xmlns:ns3="b7009bbd-f938-489b-a530-f05273710fff" xmlns:ns4="b5a44311-ed64-4a72-909f-c9dc6973bde2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ec7ca2ee893ff8a0f61d4046c6461645" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="eebd8b74-b9de-41b2-9247-c010c4973c2b"/>
@@ -11461,19 +11462,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="b5a44311-ed64-4a72-909f-c9dc6973bde2" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Description xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
-    <SortOrder xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA84097F-5807-4DCF-92C6-48C9EE26CFB8}">
   <ds:schemaRefs>
@@ -11483,6 +11471,24 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19B0E317-5E0E-4728-AB3F-40F2C2B957FB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="b5a44311-ed64-4a72-909f-c9dc6973bde2"/>
+    <ds:schemaRef ds:uri="b7009bbd-f938-489b-a530-f05273710fff"/>
+    <ds:schemaRef ds:uri="eebd8b74-b9de-41b2-9247-c010c4973c2b"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BFE547E3-BD0E-4C13-B5EC-CA56CC895052}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11500,22 +11506,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19B0E317-5E0E-4728-AB3F-40F2C2B957FB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="b5a44311-ed64-4a72-909f-c9dc6973bde2"/>
-    <ds:schemaRef ds:uri="b7009bbd-f938-489b-a530-f05273710fff"/>
-    <ds:schemaRef ds:uri="eebd8b74-b9de-41b2-9247-c010c4973c2b"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
non-functional requirement spreadsheet updates
</commit_message>
<xml_diff>
--- a/lib/davinci_crd_test_kit/requirements/cds-hooks_3.0.0-ballot_requirements.xlsx
+++ b/lib/davinci_crd_test_kit/requirements/cds-hooks_3.0.0-ballot_requirements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karlnaden/GlenViewAssociates/Inferno/source/davinci-crd-test-kit/lib/davinci_crd_test_kit/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2569BB1-4C6D-1743-87B5-05DEC082AFC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D51E2D1-0958-3C48-8D8D-671100652AEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="1320" windowWidth="33780" windowHeight="18000" activeTab="1" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
   </bookViews>
@@ -3400,9 +3400,6 @@
     <xf numFmtId="0" fontId="20" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -3417,6 +3414,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3783,14 +3783,14 @@
       <c r="C3" s="30"/>
     </row>
     <row r="4" spans="1:3" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="43" t="s">
+      <c r="A4" s="42" t="s">
         <v>291</v>
       </c>
       <c r="B4" s="31"/>
       <c r="C4" s="32"/>
     </row>
     <row r="5" spans="1:3" ht="258" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="44"/>
+      <c r="A5" s="43"/>
       <c r="B5" s="35"/>
       <c r="C5" s="30"/>
     </row>
@@ -3802,17 +3802,17 @@
       <c r="C6" s="24"/>
     </row>
     <row r="7" spans="1:3" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="45" t="s">
+      <c r="A7" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="46"/>
+      <c r="B7" s="45"/>
     </row>
     <row r="8" spans="1:3" ht="126" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="45"/>
-      <c r="B8" s="47"/>
+      <c r="A8" s="44"/>
+      <c r="B8" s="46"/>
     </row>
     <row r="9" spans="1:3" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="43"/>
+      <c r="A9" s="42"/>
       <c r="B9" s="34"/>
     </row>
     <row r="10" spans="1:3" ht="292" x14ac:dyDescent="0.2">
@@ -10962,14 +10962,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="47" t="s">
         <v>290</v>
       </c>
-      <c r="B1" s="42"/>
+      <c r="B1" s="47"/>
     </row>
     <row r="2" spans="1:2" ht="82" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="42"/>
-      <c r="B2" s="42"/>
+      <c r="A2" s="47"/>
+      <c r="B2" s="47"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="15" t="s">
@@ -11196,19 +11196,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="b5a44311-ed64-4a72-909f-c9dc6973bde2" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Description xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
-    <SortOrder xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC335ED7BB179244BF94A0DFE64544DC" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d3a0f66abe5d2a0564332877ab55d3f7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="eebd8b74-b9de-41b2-9247-c010c4973c2b" xmlns:ns3="b7009bbd-f938-489b-a530-f05273710fff" xmlns:ns4="b5a44311-ed64-4a72-909f-c9dc6973bde2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ec7ca2ee893ff8a0f61d4046c6461645" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="eebd8b74-b9de-41b2-9247-c010c4973c2b"/>
@@ -11462,6 +11449,19 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="b5a44311-ed64-4a72-909f-c9dc6973bde2" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Description xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
+    <SortOrder xmlns="eebd8b74-b9de-41b2-9247-c010c4973c2b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA84097F-5807-4DCF-92C6-48C9EE26CFB8}">
   <ds:schemaRefs>
@@ -11471,24 +11471,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19B0E317-5E0E-4728-AB3F-40F2C2B957FB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="b5a44311-ed64-4a72-909f-c9dc6973bde2"/>
-    <ds:schemaRef ds:uri="b7009bbd-f938-489b-a530-f05273710fff"/>
-    <ds:schemaRef ds:uri="eebd8b74-b9de-41b2-9247-c010c4973c2b"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BFE547E3-BD0E-4C13-B5EC-CA56CC895052}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11506,4 +11488,22 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19B0E317-5E0E-4728-AB3F-40F2C2B957FB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="b5a44311-ed64-4a72-909f-c9dc6973bde2"/>
+    <ds:schemaRef ds:uri="b7009bbd-f938-489b-a530-f05273710fff"/>
+    <ds:schemaRef ds:uri="eebd8b74-b9de-41b2-9247-c010c4973c2b"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
correct typos in requirements
</commit_message>
<xml_diff>
--- a/lib/davinci_crd_test_kit/requirements/cds-hooks_3.0.0-ballot_requirements.xlsx
+++ b/lib/davinci_crd_test_kit/requirements/cds-hooks_3.0.0-ballot_requirements.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karlnaden/GlenViewAssociates/Inferno/source/davinci-crd-test-kit/lib/davinci_crd_test_kit/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D51E2D1-0958-3C48-8D8D-671100652AEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99C0BC78-E40F-FE4E-8318-76A2E430591B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="1320" windowWidth="33780" windowHeight="18000" activeTab="1" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
   </bookViews>
@@ -5820,7 +5820,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="81" spans="1:18" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:18" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A81" s="6">
         <v>58</v>
       </c>

</xml_diff>

<commit_message>
ID-211: no custom extensions in client responses and refactor for additional tests (#133)
* correct typos in requirements

* disallow custom extensions in inferno responses

* remove conf-10 from attestations

* update requirement coverage

* thread validator through into manual checks

* fix if none exist error filter

* remove unknown extension filtering when using the no_custom_extensions validator

* request validation message filtering updates

* update structure for future tests

* revamp tagging

* update spec tests for tagging

* update requirements based on test re-org

* additional location for prefetch complete tests

* mocking bug fix for subset service on encounter-*

* update running suites against each other

* fix

* fix typos

* factor out find_completeness_tests

* restore filter

* check filtered before adding messages

* add message exclusions to no_custom_extensions validator

* bump inferno core version

* updated documentation and spec test
</commit_message>
<xml_diff>
--- a/lib/davinci_crd_test_kit/requirements/cds-hooks_3.0.0-ballot_requirements.xlsx
+++ b/lib/davinci_crd_test_kit/requirements/cds-hooks_3.0.0-ballot_requirements.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karlnaden/GlenViewAssociates/Inferno/source/davinci-crd-test-kit/lib/davinci_crd_test_kit/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D51E2D1-0958-3C48-8D8D-671100652AEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99C0BC78-E40F-FE4E-8318-76A2E430591B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="1320" windowWidth="33780" windowHeight="18000" activeTab="1" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
   </bookViews>
@@ -5820,7 +5820,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="81" spans="1:18" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:18" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A81" s="6">
         <v>58</v>
       </c>

</xml_diff>